<commit_message>
Add artist browsing, sourced album notes and remaining cover artwork
</commit_message>
<xml_diff>
--- a/data/record_collection.xlsx
+++ b/data/record_collection.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Albums" sheetId="1" r:id="Rfc5e5a39be584981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracks" sheetId="2" r:id="R346b9125d76f4a3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research_26_41" sheetId="3" r:id="R399d00c2e8644940"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Albums" sheetId="1" r:id="Rf8931e66d2164752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracks" sheetId="2" r:id="Rfe5492459f274665"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research_26_41" sheetId="3" r:id="R3224f335299f4653"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45,7 +45,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -55,6 +55,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1F4E79"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -88,7 +98,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
@@ -140,6 +150,24 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -218,8 +246,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AlbumsTable" displayName="AlbumsTable" ref="A1:AD42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="30">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AlbumsTable" displayName="AlbumsTable" ref="A1:AI42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="35">
     <x:tableColumn id="1" name="Collection ID"/>
     <x:tableColumn id="2" name="Artist (Japanese)"/>
     <x:tableColumn id="3" name="Artist (English)"/>
@@ -250,6 +278,11 @@
     <x:tableColumn id="28" name="Verification Issues"/>
     <x:tableColumn id="29" name="Verification Status"/>
     <x:tableColumn id="30" name="Last Updated"/>
+    <x:tableColumn id="31" name="Album Summary"/>
+    <x:tableColumn id="32" name="Summary Source"/>
+    <x:tableColumn id="33" name="Summary Source Label"/>
+    <x:tableColumn id="34" name="Artist Info URL"/>
+    <x:tableColumn id="35" name="Artist Info Label"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -515,101 +548,121 @@
     <x:col min="28" max="28" width="60" hidden="0" customWidth="1"/>
     <x:col min="29" max="29" width="24" hidden="0" customWidth="1"/>
     <x:col min="30" max="30" width="18" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="80" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="60" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="36" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="60" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="32" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="20" t="str">
+      <x:c r="A1" s="27" t="str">
         <x:v>Collection ID</x:v>
       </x:c>
-      <x:c r="B1" s="20" t="str">
+      <x:c r="B1" s="27" t="str">
         <x:v>Artist (Japanese)</x:v>
       </x:c>
-      <x:c r="C1" s="20" t="str">
+      <x:c r="C1" s="27" t="str">
         <x:v>Artist (English)</x:v>
       </x:c>
-      <x:c r="D1" s="20" t="str">
+      <x:c r="D1" s="27" t="str">
         <x:v>Title (Japanese)</x:v>
       </x:c>
-      <x:c r="E1" s="20" t="str">
+      <x:c r="E1" s="27" t="str">
         <x:v>Title (English)</x:v>
       </x:c>
-      <x:c r="F1" s="20" t="str">
+      <x:c r="F1" s="27" t="str">
         <x:v>Label</x:v>
       </x:c>
-      <x:c r="G1" s="20" t="str">
+      <x:c r="G1" s="27" t="str">
         <x:v>Catalog Number</x:v>
       </x:c>
-      <x:c r="H1" s="20" t="str">
+      <x:c r="H1" s="27" t="str">
         <x:v>Year</x:v>
       </x:c>
-      <x:c r="I1" s="20" t="str">
+      <x:c r="I1" s="27" t="str">
         <x:v>Format</x:v>
       </x:c>
-      <x:c r="J1" s="20" t="str">
+      <x:c r="J1" s="27" t="str">
         <x:v>Country</x:v>
       </x:c>
-      <x:c r="K1" s="20" t="str">
+      <x:c r="K1" s="27" t="str">
         <x:v>Genre</x:v>
       </x:c>
-      <x:c r="L1" s="20" t="str">
+      <x:c r="L1" s="27" t="str">
         <x:v>Retail Price (JPY)</x:v>
       </x:c>
-      <x:c r="M1" s="20" t="str">
+      <x:c r="M1" s="27" t="str">
         <x:v>Notes</x:v>
       </x:c>
-      <x:c r="N1" s="20" t="str">
+      <x:c r="N1" s="27" t="str">
         <x:v>Source Photo</x:v>
       </x:c>
-      <x:c r="O1" s="20" t="str">
+      <x:c r="O1" s="27" t="str">
         <x:v>Cover Image Filename</x:v>
       </x:c>
-      <x:c r="P1" s="20" t="str">
+      <x:c r="P1" s="27" t="str">
         <x:v>Discogs URL</x:v>
       </x:c>
-      <x:c r="Q1" s="21" t="str">
+      <x:c r="Q1" s="28" t="str">
         <x:v>Cover Source</x:v>
       </x:c>
-      <x:c r="R1" s="21" t="str">
+      <x:c r="R1" s="28" t="str">
         <x:v>Cover Status</x:v>
       </x:c>
-      <x:c r="S1" s="21" t="str">
+      <x:c r="S1" s="28" t="str">
         <x:v>Research Notes</x:v>
       </x:c>
-      <x:c r="T1" s="21" t="str">
+      <x:c r="T1" s="28" t="str">
         <x:v>Obi</x:v>
       </x:c>
-      <x:c r="U1" s="21" t="str">
+      <x:c r="U1" s="28" t="str">
         <x:v>Shelf Location</x:v>
       </x:c>
-      <x:c r="V1" s="21" t="str">
+      <x:c r="V1" s="28" t="str">
         <x:v>Vinyl Condition</x:v>
       </x:c>
-      <x:c r="W1" s="21" t="str">
+      <x:c r="W1" s="28" t="str">
         <x:v>Sleeve Condition</x:v>
       </x:c>
-      <x:c r="X1" s="21" t="str">
+      <x:c r="X1" s="28" t="str">
         <x:v>Inserts</x:v>
       </x:c>
-      <x:c r="Y1" s="21" t="str">
+      <x:c r="Y1" s="28" t="str">
         <x:v>Purchase Date</x:v>
       </x:c>
-      <x:c r="Z1" s="21" t="str">
+      <x:c r="Z1" s="28" t="str">
         <x:v>Price Paid</x:v>
       </x:c>
-      <x:c r="AA1" s="21" t="str">
+      <x:c r="AA1" s="28" t="str">
         <x:v>Purchase Currency</x:v>
       </x:c>
-      <x:c r="AB1" s="21" t="str">
+      <x:c r="AB1" s="28" t="str">
         <x:v>Verification Issues</x:v>
       </x:c>
-      <x:c r="AC1" s="21" t="str">
+      <x:c r="AC1" s="28" t="str">
         <x:v>Verification Status</x:v>
       </x:c>
-      <x:c r="AD1" s="21" t="str">
+      <x:c r="AD1" s="28" t="str">
         <x:v>Last Updated</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="90" customHeight="1">
+      <x:c r="AE1" s="28" t="str">
+        <x:v>Album Summary</x:v>
+      </x:c>
+      <x:c r="AF1" s="28" t="str">
+        <x:v>Summary Source</x:v>
+      </x:c>
+      <x:c r="AG1" s="28" t="str">
+        <x:v>Summary Source Label</x:v>
+      </x:c>
+      <x:c r="AH1" s="28" t="str">
+        <x:v>Artist Info URL</x:v>
+      </x:c>
+      <x:c r="AI1" s="28" t="str">
+        <x:v>Artist Info Label</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="120" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>01</x:v>
       </x:c>
@@ -687,8 +740,23 @@
       <x:c r="AD2" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" ht="90" customHeight="1">
+      <x:c r="AE2" s="12" t="str">
+        <x:v>A collection of enka songs with travelling and period-story themes, including “Meigetsu Akagiyama”, “Ruten” and “Akagi no Komoriuta”. The source listing documents a later export pressing of the same programme; the pressing of this copy still needs confirmation.</x:v>
+      </x:c>
+      <x:c r="AF2" s="12" t="str">
+        <x:v>https://www.discogs.com/release/5826667</x:v>
+      </x:c>
+      <x:c r="AG2" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH2" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/495700</x:v>
+      </x:c>
+      <x:c r="AI2" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="120" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>02</x:v>
       </x:c>
@@ -762,8 +830,23 @@
       <x:c r="AD3" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="90" customHeight="1">
+      <x:c r="AE3" s="12" t="str">
+        <x:v>This twelve-song collection pairs the title song with “Jūroku no Koi”, “Mineko no Komoriuta” and “Furusato Koiuta”, drawing on enka and kayōkyoku repertoire.</x:v>
+      </x:c>
+      <x:c r="AF3" s="12" t="str">
+        <x:v>https://www.discogs.com/release/7413926</x:v>
+      </x:c>
+      <x:c r="AG3" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH3" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/3756573</x:v>
+      </x:c>
+      <x:c r="AI3" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="120" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>03</x:v>
       </x:c>
@@ -804,17 +887,22 @@
       <x:c r="N4" s="6" t="str">
         <x:v>IMG_3229.jpg — bottom left</x:v>
       </x:c>
-      <x:c r="O4" s="6" t="str"/>
+      <x:c r="O4" s="6" t="str">
+        <x:v>03_reference_crop.jpg</x:v>
+      </x:c>
       <x:c r="P4" s="6" t="str">
         <x:v>https://www.discogs.com/release/9146810</x:v>
       </x:c>
-      <x:c r="Q4" s="12" t="str"/>
+      <x:c r="Q4" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3229.jpg</x:v>
+      </x:c>
       <x:c r="R4" s="12" t="str">
-        <x:v>pending</x:v>
+        <x:v>reference_photo</x:v>
       </x:c>
       <x:c r="S4" s="12" t="str">
         <x:v>Photo audit 2026-09-17: IMG_3229.jpg, bottom left. Pale sleeve with portrait in a dark kimono and sakura branches; no obi visible.
-Earlier imported notes (retained as history; may contain superseded readings): CORRECTED ID: not 石川さゆり. Cover brands「さくらの歌」; Discogs/FanFan list as「さくら貝の歌 倍賞千恵子の日本の詩」SKK-680 (1971 gatefold). No obi on this copy. Photo credit: Shinsuke Ame.</x:v>
+Earlier imported notes (retained as history; may contain superseded readings): CORRECTED ID: not 石川さゆり. Cover brands「さくらの歌」; Discogs/FanFan list as「さくら貝の歌 倍賞千恵子の日本の詩」SKK-680 (1971 gatefold). No obi on this copy. Photo credit: Shinsuke Ame.
+2026-09-17 artwork update: user authorised a straightened crop of the original reference photo while a clean online match remains unavailable.</x:v>
       </x:c>
       <x:c r="T4" s="12" t="str">
         <x:v>Not visible in supplied photo</x:v>
@@ -835,8 +923,23 @@
       <x:c r="AD4" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="90" customHeight="1">
+      <x:c r="AE4" s="12" t="str">
+        <x:v>A Japanese song collection by Chieko Baisho, presented with a cherry-blossom portrait sleeve. The photographed cover is the identification source here: its full title and exact edition still need confirmation.</x:v>
+      </x:c>
+      <x:c r="AF4" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3229.jpg</x:v>
+      </x:c>
+      <x:c r="AG4" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH4" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/575464</x:v>
+      </x:c>
+      <x:c r="AI4" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="120" customHeight="1">
       <x:c r="A5" s="6" t="str">
         <x:v>04</x:v>
       </x:c>
@@ -910,8 +1013,23 @@
       <x:c r="AD5" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="90" customHeight="1">
+      <x:c r="AE5" s="12" t="str">
+        <x:v>A twelve-track album built around songs of separation, including the title track, “Kyoto kara Hakata made” and “Ryōta no Komoriuta”. Released by RCA in 1972.</x:v>
+      </x:c>
+      <x:c r="AF5" s="12" t="str">
+        <x:v>https://www.discogs.com/release/14837576</x:v>
+      </x:c>
+      <x:c r="AG5" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH5" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/1070643</x:v>
+      </x:c>
+      <x:c r="AI5" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="120" customHeight="1">
       <x:c r="A6" s="6" t="str">
         <x:v>05</x:v>
       </x:c>
@@ -987,8 +1105,23 @@
       <x:c r="AD6" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="90" customHeight="1">
+      <x:c r="AE6" s="12" t="str">
+        <x:v>Honda’s 1971 folk and popular-song album includes “Aru Asa Umarete”, “Kibō no Kuni” and the title song “Ieji”. The sleeve presents it under the English title Going Home.</x:v>
+      </x:c>
+      <x:c r="AF6" s="12" t="str">
+        <x:v>https://www.discogs.com/release/29605807</x:v>
+      </x:c>
+      <x:c r="AG6" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH6" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/1330031</x:v>
+      </x:c>
+      <x:c r="AI6" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="120" customHeight="1">
       <x:c r="A7" s="6" t="str">
         <x:v>06</x:v>
       </x:c>
@@ -1027,17 +1160,22 @@
       <x:c r="N7" s="6" t="str">
         <x:v>IMG_3230.jpg — top right</x:v>
       </x:c>
-      <x:c r="O7" s="6" t="str"/>
+      <x:c r="O7" s="6" t="str">
+        <x:v>06_reference_crop.jpg</x:v>
+      </x:c>
       <x:c r="P7" s="6" t="str">
         <x:v>https://www.discogs.com/search/?q=%E9%83%BD%E3%81%AF%E3%82%8B%E3%81%BF%20%20%E9%83%BD%E3%81%AF%E3%82%8B%E3%81%BF%E3%81%AE%E6%B5%81%E3%81%97%E5%94%84%20/%20%E9%AD%85%E5%8A%9B%E3%81%AE%E3%81%99%E3%81%B9%E3%81%A6</x:v>
       </x:c>
-      <x:c r="Q7" s="12" t="str"/>
+      <x:c r="Q7" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3230.jpg</x:v>
+      </x:c>
       <x:c r="R7" s="12" t="str">
-        <x:v>pending</x:v>
+        <x:v>reference_photo</x:v>
       </x:c>
       <x:c r="S7" s="12" t="str">
         <x:v>Photo audit 2026-09-17: IMG_3230.jpg, top right. Red kimono portrait with red obi. A separate album from #01.
-Earlier imported notes (retained as history; may contain superseded readings): DIFFERENT from #01: red kimono close-up cover, red obi, ¥2400. Branded 流し唄 with 魅力のすべて. Full Discogs match uncertain; tracklist only partially visible on obi — DO NOT invent. Treat as separate collection entry.</x:v>
+Earlier imported notes (retained as history; may contain superseded readings): DIFFERENT from #01: red kimono close-up cover, red obi, ¥2400. Branded 流し唄 with 魅力のすべて. Full Discogs match uncertain; tracklist only partially visible on obi — DO NOT invent. Treat as separate collection entry.
+2026-09-17 artwork update: user authorised a straightened crop of the original reference photo while a clean online match remains unavailable.</x:v>
       </x:c>
       <x:c r="T7" s="12" t="str">
         <x:v>Present (visible in photo)</x:v>
@@ -1058,8 +1196,23 @@
       <x:c r="AD7" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="90" customHeight="1">
+      <x:c r="AE7" s="12" t="str">
+        <x:v>The sleeve presents this collection as Harumi Miyako’s Nagashiuta / Miryoku no Subete. Its red-kimono portrait distinguishes it from the other Nagashiuta record in this collection; the exact edition remains unidentified.</x:v>
+      </x:c>
+      <x:c r="AF7" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3230.jpg</x:v>
+      </x:c>
+      <x:c r="AG7" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH7" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/495700</x:v>
+      </x:c>
+      <x:c r="AI7" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="120" customHeight="1">
       <x:c r="A8" s="6" t="str">
         <x:v>07</x:v>
       </x:c>
@@ -1133,8 +1286,23 @@
       <x:c r="AD8" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="90" customHeight="1">
+      <x:c r="AE8" s="12" t="str">
+        <x:v>A fourteen-song selection spanning “Osaka Shigure”, “Kita no Yado kara” and “Suki ni Natta Hito”. This is the AX-7293 collection, distinct from the other Best Album sleeve on these shelves.</x:v>
+      </x:c>
+      <x:c r="AF8" s="12" t="str">
+        <x:v>https://www.discogs.com/release/19552204</x:v>
+      </x:c>
+      <x:c r="AG8" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH8" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/495700</x:v>
+      </x:c>
+      <x:c r="AI8" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="120" customHeight="1">
       <x:c r="A9" s="6" t="str">
         <x:v>08</x:v>
       </x:c>
@@ -1210,8 +1378,23 @@
       <x:c r="AD9" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="90" customHeight="1">
+      <x:c r="AE9" s="12" t="str">
+        <x:v>Sixteen enka selections, opening with “Uminari no Uta” and “Kita no Yado kara”. The programme also includes “Namida no Renrakusen” and “Anko Tsubaki wa Koi no Hana”.</x:v>
+      </x:c>
+      <x:c r="AF9" s="12" t="str">
+        <x:v>https://www.discogs.com/release/21285337</x:v>
+      </x:c>
+      <x:c r="AG9" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH9" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/495700</x:v>
+      </x:c>
+      <x:c r="AI9" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="120" customHeight="1">
       <x:c r="A10" s="6" t="str">
         <x:v>09</x:v>
       </x:c>
@@ -1285,8 +1468,23 @@
       <x:c r="AD10" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="90" customHeight="1">
+      <x:c r="AE10" s="12" t="str">
+        <x:v>A two-record selection of twenty-four songs, including “Hitorine no Komoriuta”, “Sensō wa Shiranai” and “Toki ni wa Haha no Nai Ko no Yō ni”. Released on Polydor in 1970.</x:v>
+      </x:c>
+      <x:c r="AF10" s="12" t="str">
+        <x:v>https://www.discogs.com/release/10000075</x:v>
+      </x:c>
+      <x:c r="AG10" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH10" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/66364</x:v>
+      </x:c>
+      <x:c r="AI10" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="120" customHeight="1">
       <x:c r="A11" s="6" t="str">
         <x:v>10</x:v>
       </x:c>
@@ -1358,8 +1556,23 @@
       <x:c r="AD11" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="90" customHeight="1">
+      <x:c r="AE11" s="12" t="str">
+        <x:v>A family-oriented collection of familiar international songs. Its twelve selections include “Do-Re-Mi”, “Please Mr. Postman”, “Jambalaya” and “Over the Rainbow”.</x:v>
+      </x:c>
+      <x:c r="AF11" s="12" t="str">
+        <x:v>https://www.discogs.com/release/11651826</x:v>
+      </x:c>
+      <x:c r="AG11" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH11" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/7792268</x:v>
+      </x:c>
+      <x:c r="AI11" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="120" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>11</x:v>
       </x:c>
@@ -1435,8 +1648,23 @@
       <x:c r="AD12" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="90" customHeight="1">
+      <x:c r="AE12" s="12" t="str">
+        <x:v>A twelve-song selection in CBS/Sony’s Gift Pack Series, bringing together “Shiroi Hana”, “Mimi o Sumashite Goran” and “Aki demo nai noni”.</x:v>
+      </x:c>
+      <x:c r="AF12" s="12" t="str">
+        <x:v>https://www.discogs.com/release/6410826</x:v>
+      </x:c>
+      <x:c r="AG12" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH12" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/1330031</x:v>
+      </x:c>
+      <x:c r="AI12" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="120" customHeight="1">
       <x:c r="A13" s="6" t="str">
         <x:v>12</x:v>
       </x:c>
@@ -1512,8 +1740,23 @@
       <x:c r="AD13" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="90" customHeight="1">
+      <x:c r="AE13" s="12" t="str">
+        <x:v>A collection of enduring folk songs, including “Hitori no Te”, “Tōi Sekai ni” and “Kyō no Hi wa Sayōnara”. The title track opens this 1971 CBS/Sony album.</x:v>
+      </x:c>
+      <x:c r="AF13" s="12" t="str">
+        <x:v>https://www.discogs.com/release/14124740</x:v>
+      </x:c>
+      <x:c r="AG13" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH13" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/1330031</x:v>
+      </x:c>
+      <x:c r="AI13" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="120" customHeight="1">
       <x:c r="A14" s="6" t="str">
         <x:v>13</x:v>
       </x:c>
@@ -1550,17 +1793,22 @@
       <x:c r="N14" s="6" t="str">
         <x:v>IMG_3236.jpg — top left</x:v>
       </x:c>
-      <x:c r="O14" s="6" t="str"/>
+      <x:c r="O14" s="6" t="str">
+        <x:v>13_reference_crop.jpg</x:v>
+      </x:c>
       <x:c r="P14" s="6" t="str">
         <x:v>https://www.discogs.com/search/?q=%E5%AE%AE%E5%9F%8E%E9%81%93%E9%9B%84%EF%BC%88%E4%BD%9C%E5%93%81%EF%BC%89%EF%BC%8F%E6%BC%94%E5%A5%8F%EF%BC%9A%E5%AE%AE%E5%9F%8E%E5%96%9C%E4%BB%A3%E5%AD%90%E3%83%BB%E5%AE%AE%E5%9F%8E%E6%95%B0%E6%B1%9F%E3%83%BB%E4%BC%8A%E8%97%A4%E4%BA%AC%E5%AD%90%20%E4%BB%96%20SJL-2080%20%E7%AE%8F%20%E5%90%8D%E6%9B%B2%E3%81%AE%E8%AA%BF%E3%81%B9%E3%80%883%E3%80%89%EF%BC%8F%E5%AE%AE%E5%9F%8E%E9%81%93%E9%9B%84%E4%BD%9C%E5%93%81%E9%9B%86</x:v>
       </x:c>
-      <x:c r="Q14" s="12" t="str"/>
+      <x:c r="Q14" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3236.jpg</x:v>
+      </x:c>
       <x:c r="R14" s="12" t="str">
-        <x:v>pending</x:v>
+        <x:v>reference_photo</x:v>
       </x:c>
       <x:c r="S14" s="12" t="str">
         <x:v>Photo audit 2026-09-17: IMG_3236.jpg, top left. Artist, title and visible catalogue identifier checked against the original photograph.
-Earlier imported notes (retained as history; may contain superseded readings): Jacket clearly prints SJL-2080 (not SJ-3008-3). Performers on jacket: 宮城喜代子(箏), 宮城数江(唄・箏), 伊藤京子(唄)他. 'KOTO music' branding. Pieces listed on front.</x:v>
+Earlier imported notes (retained as history; may contain superseded readings): Jacket clearly prints SJL-2080 (not SJ-3008-3). Performers on jacket: 宮城喜代子(箏), 宮城数江(唄・箏), 伊藤京子(唄)他. 'KOTO music' branding. Pieces listed on front.
+2026-09-17 artwork update: user authorised a straightened crop of the original reference photo while a clean online match remains unavailable.</x:v>
       </x:c>
       <x:c r="T14" s="12" t="str">
         <x:v>Not visible in supplied photo</x:v>
@@ -1581,8 +1829,23 @@
       <x:c r="AD14" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15" ht="90" customHeight="1">
+      <x:c r="AE14" s="12" t="str">
+        <x:v>Volume three of a koto collection devoted to compositions by Michio Miyagi. The sleeve credits performers including Kiyoko Miyagi and Kazue Miyagi, and lists “Haru no Umi” among the works.</x:v>
+      </x:c>
+      <x:c r="AF14" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3236.jpg</x:v>
+      </x:c>
+      <x:c r="AG14" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH14" s="12" t="str">
+        <x:v>https://en.wikipedia.org/wiki/Michio_Miyagi</x:v>
+      </x:c>
+      <x:c r="AI14" s="12" t="str">
+        <x:v>Wikipedia</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="120" customHeight="1">
       <x:c r="A15" s="6" t="str">
         <x:v>14</x:v>
       </x:c>
@@ -1656,8 +1919,23 @@
       <x:c r="AD15" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="90" customHeight="1">
+      <x:c r="AE15" s="12" t="str">
+        <x:v>A selection of twelve songs, including “Jūsan’ya”, “Atooi Shamisen”, “Gion Kouta” and “Tenryū Kudareba”. The programme draws on Japanese traditional and popular-song repertoire.</x:v>
+      </x:c>
+      <x:c r="AF15" s="12" t="str">
+        <x:v>https://www.discogs.com/release/10151877</x:v>
+      </x:c>
+      <x:c r="AG15" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH15" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/7511264</x:v>
+      </x:c>
+      <x:c r="AI15" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="120" customHeight="1">
       <x:c r="A16" s="6" t="str">
         <x:v>15</x:v>
       </x:c>
@@ -1729,8 +2007,23 @@
       <x:c r="AD16" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" ht="90" customHeight="1">
+      <x:c r="AE16" s="12" t="str">
+        <x:v>Released on 5 March 1971, this is the third album in Sony’s official Red Birds discography. It sits between Red Birds and Takeda no Komoriuta in the group’s early recording history.</x:v>
+      </x:c>
+      <x:c r="AF16" s="12" t="str">
+        <x:v>https://www.sonymusic.co.jp/Music/Info/junkoyamamoto/akaitoridisc.html</x:v>
+      </x:c>
+      <x:c r="AG16" s="12" t="str">
+        <x:v>Sony Music discography</x:v>
+      </x:c>
+      <x:c r="AH16" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/2812156</x:v>
+      </x:c>
+      <x:c r="AI16" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="120" customHeight="1">
       <x:c r="A17" s="6" t="str">
         <x:v>16</x:v>
       </x:c>
@@ -1805,8 +2098,23 @@
       <x:c r="AD17" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="90" customHeight="1">
+      <x:c r="AE17" s="12" t="str">
+        <x:v>Originally released on 10 April 1978, this nine-track album opens with the spoken “Genki Desu ka” and includes “Wakareuta”, “Keshō” and “Sejō”. This collection holds the C28A0146 reissue; its pressing date is still unconfirmed.</x:v>
+      </x:c>
+      <x:c r="AF17" s="12" t="str">
+        <x:v>https://www.yamahamusic.co.jp/s/ymc/discography/266?ima=0000&amp;link=ROBO004</x:v>
+      </x:c>
+      <x:c r="AG17" s="12" t="str">
+        <x:v>Yamaha Music album notes</x:v>
+      </x:c>
+      <x:c r="AH17" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/1082785</x:v>
+      </x:c>
+      <x:c r="AI17" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="120" customHeight="1">
       <x:c r="A18" s="6" t="str">
         <x:v>17</x:v>
       </x:c>
@@ -1882,8 +2190,23 @@
       <x:c r="AD18" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="90" customHeight="1">
+      <x:c r="AE18" s="12" t="str">
+        <x:v>Iruka’s JULIA is represented here by the PANAM GWP-1019 LP. The artist’s official discography documents the album alongside her wider recording catalogue.</x:v>
+      </x:c>
+      <x:c r="AF18" s="12" t="str">
+        <x:v>https://www.crownrecord.co.jp/s/c01/artist/iruka/discography</x:v>
+      </x:c>
+      <x:c r="AG18" s="12" t="str">
+        <x:v>Nippon Crown discography</x:v>
+      </x:c>
+      <x:c r="AH18" s="12" t="str">
+        <x:v>https://www.crownrecord.co.jp/s/c01/artist/iruka/discography</x:v>
+      </x:c>
+      <x:c r="AI18" s="12" t="str">
+        <x:v>Official artist page</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="120" customHeight="1">
       <x:c r="A19" s="6" t="str">
         <x:v>18</x:v>
       </x:c>
@@ -1957,8 +2280,23 @@
       <x:c r="AD19" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="20" ht="90" customHeight="1">
+      <x:c r="AE19" s="12" t="str">
+        <x:v>A twelve-song folk album by Wish, ending with “Rokugatsu no Komoriuta”. Other selections include “Kazaguruma”, “Tegami” and “Shihatsu Ressha de”.</x:v>
+      </x:c>
+      <x:c r="AF19" s="12" t="str">
+        <x:v>https://www.discogs.com/release/15856177</x:v>
+      </x:c>
+      <x:c r="AG19" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH19" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/6163738</x:v>
+      </x:c>
+      <x:c r="AI19" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="120" customHeight="1">
       <x:c r="A20" s="6" t="str">
         <x:v>19</x:v>
       </x:c>
@@ -2032,8 +2370,23 @@
       <x:c r="AD20" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21" ht="90" customHeight="1">
+      <x:c r="AE20" s="12" t="str">
+        <x:v>A ten-song album from 1983, closing with its title song, “Umi no Mieru Heya”. The programme also includes “Watashi wa Ima”, “Shabon-dama” and “Room Mirror”.</x:v>
+      </x:c>
+      <x:c r="AF20" s="12" t="str">
+        <x:v>https://www.discogs.com/release/16035381</x:v>
+      </x:c>
+      <x:c r="AG20" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH20" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/7500205</x:v>
+      </x:c>
+      <x:c r="AI20" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="120" customHeight="1">
       <x:c r="A21" s="6" t="str">
         <x:v>20</x:v>
       </x:c>
@@ -2107,8 +2460,23 @@
       <x:c r="AD21" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="22" ht="90" customHeight="1">
+      <x:c r="AE21" s="12" t="str">
+        <x:v>The Columbia sleeve identifies this as Chiyoko Shimakura’s Aishōshū, a collection of favourite songs. The visible catalogue number is ALS-5027; the release year still needs confirmation.</x:v>
+      </x:c>
+      <x:c r="AF21" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3237.jpg</x:v>
+      </x:c>
+      <x:c r="AG21" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH21" s="12" t="str">
+        <x:v>https://en.wikipedia.org/wiki/Chiyoko_Shimakura</x:v>
+      </x:c>
+      <x:c r="AI21" s="12" t="str">
+        <x:v>Wikipedia</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="120" customHeight="1">
       <x:c r="A22" s="6" t="str">
         <x:v>21</x:v>
       </x:c>
@@ -2182,8 +2550,23 @@
       <x:c r="AD22" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="23" ht="90" customHeight="1">
+      <x:c r="AE22" s="12" t="str">
+        <x:v>A vocal jazz set mixing standards and contemporary songs, from “How About You?” and “These Foolish Things” to Stevie Wonder’s “Too Shy to Say”. Released by Philips in 1980.</x:v>
+      </x:c>
+      <x:c r="AF22" s="12" t="str">
+        <x:v>https://www.discogs.com/release/4576441</x:v>
+      </x:c>
+      <x:c r="AG22" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH22" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/2762163</x:v>
+      </x:c>
+      <x:c r="AI22" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="120" customHeight="1">
       <x:c r="A23" s="6" t="str">
         <x:v>22</x:v>
       </x:c>
@@ -2257,8 +2640,23 @@
       <x:c r="AD23" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="24" ht="90" customHeight="1">
+      <x:c r="AE23" s="12" t="str">
+        <x:v>This two-record collection gathers twenty-four songs, including “Jūshichi no Natsu”, “Hajimete no Dekigoto” and “Watashi no Aoi Tori”. It is Junko Sakurada’s edition of Victor’s Best Collection ’76 series.</x:v>
+      </x:c>
+      <x:c r="AF23" s="12" t="str">
+        <x:v>https://www.discogs.com/release/7643818</x:v>
+      </x:c>
+      <x:c r="AG23" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH23" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/3390757</x:v>
+      </x:c>
+      <x:c r="AI23" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="120" customHeight="1">
       <x:c r="A24" s="6" t="str">
         <x:v>23</x:v>
       </x:c>
@@ -2336,8 +2734,23 @@
       <x:c r="AD24" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="25" ht="90" customHeight="1">
+      <x:c r="AE24" s="12" t="str">
+        <x:v>A two-record Ayumi Ishida collection in Columbia’s Green &amp; Glorious 3000 series. The obi advertises songs including “Blue Light Yokohama” and “Taiyō wa Naiteiru”.</x:v>
+      </x:c>
+      <x:c r="AF24" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3238.jpg</x:v>
+      </x:c>
+      <x:c r="AG24" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH24" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/311861</x:v>
+      </x:c>
+      <x:c r="AI24" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="120" customHeight="1">
       <x:c r="A25" s="6" t="str">
         <x:v>24</x:v>
       </x:c>
@@ -2374,17 +2787,22 @@
       <x:c r="N25" s="6" t="str">
         <x:v>IMG_3238.jpg — bottom right</x:v>
       </x:c>
-      <x:c r="O25" s="6" t="str"/>
+      <x:c r="O25" s="6" t="str">
+        <x:v>24_reference_crop.jpg</x:v>
+      </x:c>
       <x:c r="P25" s="6" t="str">
         <x:v>https://www.discogs.com/search/?q=%E9%83%BD%E3%81%AF%E3%82%8B%E3%81%BF%20%20%E3%83%99%E3%82%B9%E3%83%88%E3%82%A2%E3%83%AB%E3%83%90%E3%83%A0</x:v>
       </x:c>
-      <x:c r="Q25" s="12" t="str"/>
+      <x:c r="Q25" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3238.jpg</x:v>
+      </x:c>
       <x:c r="R25" s="12" t="str">
-        <x:v>pending</x:v>
+        <x:v>reference_photo</x:v>
       </x:c>
       <x:c r="S25" s="12" t="str">
         <x:v>Photo audit 2026-09-17: IMG_3238.jpg, bottom right. Cream kimono, peach background and blue sakura border. Separate from #07.
-Earlier imported notes (retained as history; may contain superseded readings): DISTINCT from #07 and #08. Cream/off-white kimono, peach background, navy blue sakura border, vertical red title panel. Catalog number not visible on front crop. Tracklist unverified for this specific jacket — incomplete.</x:v>
+Earlier imported notes (retained as history; may contain superseded readings): DISTINCT from #07 and #08. Cream/off-white kimono, peach background, navy blue sakura border, vertical red title panel. Catalog number not visible on front crop. Tracklist unverified for this specific jacket — incomplete.
+2026-09-17 artwork update: user authorised a straightened crop of the original reference photo while a clean online match remains unavailable.</x:v>
       </x:c>
       <x:c r="T25" s="12" t="str">
         <x:v>Not visible in supplied photo</x:v>
@@ -2405,8 +2823,23 @@
       <x:c r="AD25" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="26" ht="90" customHeight="1">
+      <x:c r="AE25" s="12" t="str">
+        <x:v>A Harumi Miyako compilation titled Best Album, identifiable here by its blue blossom border. Its precise catalogue number and programme still need checking, so it is kept separate from the AX-7293 compilation.</x:v>
+      </x:c>
+      <x:c r="AF25" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3238.jpg</x:v>
+      </x:c>
+      <x:c r="AG25" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH25" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/495700</x:v>
+      </x:c>
+      <x:c r="AI25" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="120" customHeight="1">
       <x:c r="A26" s="6" t="str">
         <x:v>25</x:v>
       </x:c>
@@ -2480,8 +2913,23 @@
       <x:c r="AD26" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="27" ht="90" customHeight="1">
+      <x:c r="AE26" s="12" t="str">
+        <x:v>A twenty-four-song, two-record anthology including “Coffee Rumba”, “Tokyo Blues” and “Akashia no Ame ga Yamu Toki”. The title translates approximately as Love, Affection, and Tears.</x:v>
+      </x:c>
+      <x:c r="AF26" s="12" t="str">
+        <x:v>https://www.discogs.com/release/11645824</x:v>
+      </x:c>
+      <x:c r="AG26" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH26" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/1088200</x:v>
+      </x:c>
+      <x:c r="AI26" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="120" customHeight="1">
       <x:c r="A27" s="6" t="str">
         <x:v>26</x:v>
       </x:c>
@@ -2555,8 +3003,23 @@
       <x:c r="AD27" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="28" ht="90" customHeight="1">
+      <x:c r="AE27" s="12" t="str">
+        <x:v>A lullaby programme combining Japanese songs with international selections such as “Hushabye Mountain”, “Summertime” and “Hush Little Baby”. Released on Philips in 1968.</x:v>
+      </x:c>
+      <x:c r="AF27" s="12" t="str">
+        <x:v>https://www.discogs.com/release/14059461</x:v>
+      </x:c>
+      <x:c r="AG27" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH27" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/440134</x:v>
+      </x:c>
+      <x:c r="AI27" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="120" customHeight="1">
       <x:c r="A28" s="6" t="str">
         <x:v>27</x:v>
       </x:c>
@@ -2630,8 +3093,23 @@
       <x:c r="AD28" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="29" ht="90" customHeight="1">
+      <x:c r="AE28" s="12" t="str">
+        <x:v>Yamagata’s debut album, originally released on 25 March 1973 when she was sixteen. Its folk repertoire includes “Kaze ni Fukarete Ikō”, “Akai Hana Shiroi Hana” and “Mayonaka no Guitar”.</x:v>
+      </x:c>
+      <x:c r="AF28" s="12" t="str">
+        <x:v>https://columbia.jp/artist-info/yamagatasumiko/discography/COCP-39360.html</x:v>
+      </x:c>
+      <x:c r="AG28" s="12" t="str">
+        <x:v>Columbia album notes</x:v>
+      </x:c>
+      <x:c r="AH28" s="12" t="str">
+        <x:v>https://columbia.jp/j-digs/artists/sumikoyamagata.html</x:v>
+      </x:c>
+      <x:c r="AI28" s="12" t="str">
+        <x:v>Columbia artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="120" customHeight="1">
       <x:c r="A29" s="6" t="str">
         <x:v>28</x:v>
       </x:c>
@@ -2705,8 +3183,23 @@
       <x:c r="AD29" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="30" ht="90" customHeight="1">
+      <x:c r="AE29" s="12" t="str">
+        <x:v>Recorded at Tokyo’s Sankei Hall on 27 October 1969, this recital pairs Ishida’s songs with film themes and international favourites. Selections include “Blue Light Yokohama”, “Scarborough Fair” and “The Shadow of Your Smile”.</x:v>
+      </x:c>
+      <x:c r="AF29" s="12" t="str">
+        <x:v>https://www.discogs.com/release/5305338</x:v>
+      </x:c>
+      <x:c r="AG29" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH29" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/311861</x:v>
+      </x:c>
+      <x:c r="AI29" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="120" customHeight="1">
       <x:c r="A30" s="6" t="str">
         <x:v>29</x:v>
       </x:c>
@@ -2782,8 +3275,23 @@
       <x:c r="AD30" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="31" ht="90" customHeight="1">
+      <x:c r="AE30" s="12" t="str">
+        <x:v>Nishida interprets twelve Japanese lyrical songs, including “Hamabe no Uta”, “Kōjō no Tsuki”, “Hana” and the title piece. The collection was issued by Polydor in 1970.</x:v>
+      </x:c>
+      <x:c r="AF30" s="12" t="str">
+        <x:v>https://www.discogs.com/release/35741143</x:v>
+      </x:c>
+      <x:c r="AG30" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH30" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/1088200</x:v>
+      </x:c>
+      <x:c r="AI30" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="120" customHeight="1">
       <x:c r="A31" s="6" t="str">
         <x:v>30</x:v>
       </x:c>
@@ -2857,8 +3365,23 @@
       <x:c r="AD31" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="32" ht="90" customHeight="1">
+      <x:c r="AE31" s="12" t="str">
+        <x:v>An enka album led by “Omoide-zake”, alongside interpretations of “Tsugaru Kaikyō Fuyugeshiki”, “Kita no Yado kara” and “Kitaguni no Haru”. Released in 1979.</x:v>
+      </x:c>
+      <x:c r="AF31" s="12" t="str">
+        <x:v>https://www.discogs.com/release/9432885</x:v>
+      </x:c>
+      <x:c r="AG31" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH31" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/5666652</x:v>
+      </x:c>
+      <x:c r="AI31" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="120" customHeight="1">
       <x:c r="A32" s="6" t="str">
         <x:v>31</x:v>
       </x:c>
@@ -2932,8 +3455,23 @@
       <x:c r="AD32" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="33" ht="90" customHeight="1">
+      <x:c r="AE32" s="12" t="str">
+        <x:v>The second volume of Uta wa Waga Inochi, presented in a blue Columbia sleeve. The photographed copy identifies Hibari Misora and catalogue ALS-5059; the sleeve is retained as the primary identification source.</x:v>
+      </x:c>
+      <x:c r="AF32" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3233.jpg</x:v>
+      </x:c>
+      <x:c r="AG32" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH32" s="12" t="str">
+        <x:v>https://en.wikipedia.org/wiki/Hibari_Misora</x:v>
+      </x:c>
+      <x:c r="AI32" s="12" t="str">
+        <x:v>Wikipedia</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="120" customHeight="1">
       <x:c r="A33" s="6" t="str">
         <x:v>32</x:v>
       </x:c>
@@ -3007,8 +3545,23 @@
       <x:c r="AD33" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="34" ht="90" customHeight="1">
+      <x:c r="AE33" s="12" t="str">
+        <x:v>A Victor album bearing the title “Anata ni Ageru”. The photographed sleeve confirms Mineko Nishikawa and catalogue SJX-198, with a close-up portrait and pink title panel.</x:v>
+      </x:c>
+      <x:c r="AF33" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3233.jpg</x:v>
+      </x:c>
+      <x:c r="AG33" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH33" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/3756573</x:v>
+      </x:c>
+      <x:c r="AI33" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="120" customHeight="1">
       <x:c r="A34" s="6" t="str">
         <x:v>33</x:v>
       </x:c>
@@ -3049,17 +3602,23 @@
       <x:c r="N34" s="6" t="str">
         <x:v>IMG_3233.jpg — bottom right</x:v>
       </x:c>
-      <x:c r="O34" s="6" t="str"/>
+      <x:c r="O34" s="6" t="str">
+        <x:v>33_official_front.jpg</x:v>
+      </x:c>
       <x:c r="P34" s="6" t="str">
         <x:v>https://www.discogs.com/search/?q=%E9%83%BD%E3%81%AF%E3%82%8B%E3%81%BF%20AX-7226%20%E5%A4%A7%E9%98%AA%E3%81%97%E3%81%90%E3%82%8C</x:v>
       </x:c>
-      <x:c r="Q34" s="12" t="str"/>
+      <x:c r="Q34" s="12" t="str">
+        <x:v>https://columbia.jp/artist-info/harumi/discography/COKM-46459.html</x:v>
+      </x:c>
       <x:c r="R34" s="12" t="str">
-        <x:v>pending</x:v>
+        <x:v>official</x:v>
       </x:c>
       <x:c r="S34" s="12" t="str">
         <x:v>Photo audit 2026-09-17: IMG_3233.jpg, bottom right. AX-7226 is printed at the top right; the prior AK-7168 reading was incorrect.
-Earlier imported notes (retained as history; may contain superseded readings): Green vertical banner lists tracks matching Columbia album AX-7226 (1980-02-25). Photo tentatively read AK-7168 (AK-216 is the single). Prefer official AX-7226; verify spine/label. 12 tracks.</x:v>
+Earlier imported notes (retained as history; may contain superseded readings): Green vertical banner lists tracks matching Columbia album AX-7226 (1980-02-25). Photo tentatively read AK-7168 (AK-216 is the single). Prefer official AX-7226; verify spine/label. 12 tracks.
+2026-09-17 artwork update: user authorised a straightened crop of the original reference photo while a clean online match remains unavailable.
+Clean matching front cover sourced from Columbia: https://columbia.jp/artist-info/jacket/COKM-46459.jpg. Original LP date 1980-02-25; the 2026 date on the page is the digital reissue.</x:v>
       </x:c>
       <x:c r="T34" s="12" t="str">
         <x:v>Present (visible in photo)</x:v>
@@ -3078,8 +3637,23 @@
       <x:c r="AD34" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="35" ht="90" customHeight="1">
+      <x:c r="AE34" s="12" t="str">
+        <x:v>Originally issued on 25 February 1980, this twelve-song album opens with “Osaka Shigure” and includes “Sayonara Kaikyō” and “Harumi”. Columbia’s official reissue page confirms the original AX-7226 catalogue number.</x:v>
+      </x:c>
+      <x:c r="AF34" s="12" t="str">
+        <x:v>https://columbia.jp/artist-info/harumi/discography/COKM-46459.html</x:v>
+      </x:c>
+      <x:c r="AG34" s="12" t="str">
+        <x:v>Columbia album notes</x:v>
+      </x:c>
+      <x:c r="AH34" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/495700</x:v>
+      </x:c>
+      <x:c r="AI34" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="120" customHeight="1">
       <x:c r="A35" s="6" t="str">
         <x:v>34</x:v>
       </x:c>
@@ -3118,17 +3692,22 @@
       <x:c r="N35" s="6" t="str">
         <x:v>IMG_3234.jpg — top left</x:v>
       </x:c>
-      <x:c r="O35" s="6" t="str"/>
+      <x:c r="O35" s="6" t="str">
+        <x:v>34_reference_crop.jpg</x:v>
+      </x:c>
       <x:c r="P35" s="6" t="str">
         <x:v>https://www.discogs.com/search/?q=%E8%A5%BF%E5%B7%9D%E5%B3%B0%E5%AD%90%20SJV-836~7%20%E3%83%99%E3%82%B9%E3%83%88%E3%83%BB%E3%82%B3%E3%83%AC%E3%82%AF%E3%82%B7%E3%83%A7%E3%83%B3%20%2776</x:v>
       </x:c>
-      <x:c r="Q35" s="12" t="str"/>
+      <x:c r="Q35" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3234.jpg</x:v>
+      </x:c>
       <x:c r="R35" s="12" t="str">
-        <x:v>pending</x:v>
+        <x:v>reference_photo</x:v>
       </x:c>
       <x:c r="S35" s="12" t="str">
         <x:v>Photo audit 2026-09-17: IMG_3234.jpg, top left. Victor two-record set. Catalogue SJV-836~7 is visible on the sleeve.
-Earlier imported notes (retained as history; may contain superseded readings): Victor SJV-836~7 confirmed. Distinct from #22 Sakurada SJV-832~3. Parent SXV-8002 incorrect.</x:v>
+Earlier imported notes (retained as history; may contain superseded readings): Victor SJV-836~7 confirmed. Distinct from #22 Sakurada SJV-832~3. Parent SXV-8002 incorrect.
+2026-09-17 artwork update: user authorised a straightened crop of the original reference photo while a clean online match remains unavailable.</x:v>
       </x:c>
       <x:c r="T35" s="12" t="str">
         <x:v>Not visible in supplied photo</x:v>
@@ -3149,8 +3728,23 @@
       <x:c r="AD35" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="36" ht="90" customHeight="1">
+      <x:c r="AE35" s="12" t="str">
+        <x:v>Mineko Nishikawa’s two-record contribution to Victor’s Best Collection ’76 series. Its SJV-836–7 catalogue number distinguishes it from Junko Sakurada’s similarly titled set.</x:v>
+      </x:c>
+      <x:c r="AF35" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3234.jpg</x:v>
+      </x:c>
+      <x:c r="AG35" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH35" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/3756573</x:v>
+      </x:c>
+      <x:c r="AI35" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="120" customHeight="1">
       <x:c r="A36" s="6" t="str">
         <x:v>35</x:v>
       </x:c>
@@ -3223,8 +3817,23 @@
       <x:c r="AD36" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="37" ht="90" customHeight="1">
+      <x:c r="AE36" s="12" t="str">
+        <x:v>A twelve-track collection led by “Kanashimi no Machi”, with “Onna no Melody” and “Ai no Kodoku”. This RCA issue uses the CD-4 four-channel format advertised as QuadraDisc on the sleeve.</x:v>
+      </x:c>
+      <x:c r="AF36" s="12" t="str">
+        <x:v>https://www.discogs.com/release/15416408</x:v>
+      </x:c>
+      <x:c r="AG36" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH36" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/1070643</x:v>
+      </x:c>
+      <x:c r="AI36" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="120" customHeight="1">
       <x:c r="A37" s="6" t="str">
         <x:v>36</x:v>
       </x:c>
@@ -3298,8 +3907,23 @@
       <x:c r="AD37" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="38" ht="90" customHeight="1">
+      <x:c r="AE37" s="12" t="str">
+        <x:v>A two-record Hibari Misora collection in the Golden Star Deluxe series. The photographed sleeve confirms AB-7001–2; the detailed programme is awaiting verification rather than borrowing another singer’s track list.</x:v>
+      </x:c>
+      <x:c r="AF37" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3234.jpg</x:v>
+      </x:c>
+      <x:c r="AG37" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH37" s="12" t="str">
+        <x:v>https://en.wikipedia.org/wiki/Hibari_Misora</x:v>
+      </x:c>
+      <x:c r="AI37" s="12" t="str">
+        <x:v>Wikipedia</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="120" customHeight="1">
       <x:c r="A38" s="6" t="str">
         <x:v>37</x:v>
       </x:c>
@@ -3336,15 +3960,20 @@
       <x:c r="N38" s="6" t="str">
         <x:v>IMG_3234.jpg — bottom right</x:v>
       </x:c>
-      <x:c r="O38" s="6" t="str"/>
+      <x:c r="O38" s="6" t="str">
+        <x:v>37_reference_crop.jpg</x:v>
+      </x:c>
       <x:c r="P38" s="6" t="str"/>
-      <x:c r="Q38" s="12" t="str"/>
+      <x:c r="Q38" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3234.jpg</x:v>
+      </x:c>
       <x:c r="R38" s="12" t="str">
-        <x:v>pending</x:v>
+        <x:v>reference_photo</x:v>
       </x:c>
       <x:c r="S38" s="12" t="str">
         <x:v>Photo audit 2026-09-17: IMG_3234.jpg, bottom right. Sony SQ four-channel sampler with black concentric-groove artwork. SPEC-94019 is a candidate, not a photo-confirmed identifier.
-Earlier imported notes (retained as history; may contain superseded readings): Black groove-art cover; bottom text 地球はひとつ SQ 4チャンネル; Sony + SX-1318 on jacket. SQ 4-channel demo/sampler known for including 原信夫とシャープス＆フラッツ「Bitter Sweet Samba」. Full side-assigned tracklist not verified without inventing — omit tracks.</x:v>
+Earlier imported notes (retained as history; may contain superseded readings): Black groove-art cover; bottom text 地球はひとつ SQ 4チャンネル; Sony + SX-1318 on jacket. SQ 4-channel demo/sampler known for including 原信夫とシャープス＆フラッツ「Bitter Sweet Samba」. Full side-assigned tracklist not verified without inventing — omit tracks.
+2026-09-17 artwork update: user authorised a straightened crop of the original reference photo while a clean online match remains unavailable.</x:v>
       </x:c>
       <x:c r="T38" s="12" t="str">
         <x:v>Not visible in supplied photo</x:v>
@@ -3365,8 +3994,19 @@
       <x:c r="AD38" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="39" ht="90" customHeight="1">
+      <x:c r="AE38" s="12" t="str">
+        <x:v>A Sony demonstration record promoting SQ four-channel sound, under the title Chikyū wa Hitotsu (“The Earth Is One”). The exact edition and performers are still being checked.</x:v>
+      </x:c>
+      <x:c r="AF38" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3234.jpg</x:v>
+      </x:c>
+      <x:c r="AG38" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH38" s="12" t="str"/>
+      <x:c r="AI38" s="12" t="str"/>
+    </x:row>
+    <x:row r="39" ht="120" customHeight="1">
       <x:c r="A39" s="6" t="str">
         <x:v>38</x:v>
       </x:c>
@@ -3440,8 +4080,23 @@
       <x:c r="AD39" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="40" ht="90" customHeight="1">
+      <x:c r="AE39" s="12" t="str">
+        <x:v>Sony’s official discography dates Studio Live to 20 December 1971, following Takeda no Komoriuta. It is an early Red Birds release, distinct from the later Million People concert album.</x:v>
+      </x:c>
+      <x:c r="AF39" s="12" t="str">
+        <x:v>https://www.sonymusic.co.jp/Music/Info/junkoyamamoto/akaitoridisc.html</x:v>
+      </x:c>
+      <x:c r="AG39" s="12" t="str">
+        <x:v>Sony Music discography</x:v>
+      </x:c>
+      <x:c r="AH39" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/2812156</x:v>
+      </x:c>
+      <x:c r="AI39" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="120" customHeight="1">
       <x:c r="A40" s="6" t="str">
         <x:v>39</x:v>
       </x:c>
@@ -3480,17 +4135,22 @@
       <x:c r="N40" s="6" t="str">
         <x:v>IMG_3235.jpg — top right</x:v>
       </x:c>
-      <x:c r="O40" s="6" t="str"/>
+      <x:c r="O40" s="6" t="str">
+        <x:v>39_reference_crop.jpg</x:v>
+      </x:c>
       <x:c r="P40" s="6" t="str">
         <x:v>https://www.discogs.com/search/?q=%E8%B5%A4%E3%81%84%E9%B3%A5%20ETP-60223~24%20%E3%82%B4%E3%83%BC%E3%83%AB%E3%83%87%E3%83%B3%E3%83%BB%E3%83%87%E3%82%A3%E3%82%B9%E3%82%AF</x:v>
       </x:c>
-      <x:c r="Q40" s="12" t="str"/>
+      <x:c r="Q40" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3235.jpg</x:v>
+      </x:c>
       <x:c r="R40" s="12" t="str">
-        <x:v>pending</x:v>
+        <x:v>reference_photo</x:v>
       </x:c>
       <x:c r="S40" s="12" t="str">
         <x:v>Photo audit 2026-09-17: IMG_3235.jpg, top right. Orange-bordered two-record set. The visible ¥380 sticker is a shop price, not a confirmed purchase price.
-Earlier imported notes (retained as history; may contain superseded readings): Jacket shows ETP-60223~24 (parent ETP-60222~23). Orange-border 2LP group photo.</x:v>
+Earlier imported notes (retained as history; may contain superseded readings): Jacket shows ETP-60223~24 (parent ETP-60222~23). Orange-border 2LP group photo.
+2026-09-17 artwork update: user authorised a straightened crop of the original reference photo while a clean online match remains unavailable.</x:v>
       </x:c>
       <x:c r="T40" s="12" t="str">
         <x:v>Not visible in supplied photo</x:v>
@@ -3511,8 +4171,23 @@
       <x:c r="AD40" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="41" ht="90" customHeight="1">
+      <x:c r="AE40" s="12" t="str">
+        <x:v>A two-record Red Birds compilation issued as Golden Disk. The orange-bordered sleeve identifies catalogue ETP-60223–24; its release year remains unconfirmed.</x:v>
+      </x:c>
+      <x:c r="AF40" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3235.jpg</x:v>
+      </x:c>
+      <x:c r="AG40" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH40" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/2812156</x:v>
+      </x:c>
+      <x:c r="AI40" s="12" t="str">
+        <x:v>Discogs artist profile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="120" customHeight="1">
       <x:c r="A41" s="6" t="str">
         <x:v>40</x:v>
       </x:c>
@@ -3549,15 +4224,20 @@
       <x:c r="N41" s="6" t="str">
         <x:v>IMG_3235.jpg — bottom left</x:v>
       </x:c>
-      <x:c r="O41" s="6" t="str"/>
+      <x:c r="O41" s="6" t="str">
+        <x:v>40_reference_crop.jpg</x:v>
+      </x:c>
       <x:c r="P41" s="6" t="str"/>
-      <x:c r="Q41" s="12" t="str"/>
+      <x:c r="Q41" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3235.jpg</x:v>
+      </x:c>
       <x:c r="R41" s="12" t="str">
-        <x:v>pending</x:v>
+        <x:v>reference_photo</x:v>
       </x:c>
       <x:c r="S41" s="12" t="str">
         <x:v>Photo audit 2026-09-17: IMG_3235.jpg, bottom left. The sleeve reads 笹川鎮江 愛吟集 第2集. Smaller-format sleeve with moon and blossoms.
-Earlier imported notes (retained as history; may contain superseded readings): Moon &amp; sakura 愛吟集 第2集. Discogs SJX-10115 is 浜口庫之助 雨のピエロ — catalog collision; do not use. Jacket catalog unconfirmed on crop.</x:v>
+Earlier imported notes (retained as history; may contain superseded readings): Moon &amp; sakura 愛吟集 第2集. Discogs SJX-10115 is 浜口庫之助 雨のピエロ — catalog collision; do not use. Jacket catalog unconfirmed on crop.
+2026-09-17 artwork update: user authorised a straightened crop of the original reference photo while a clean online match remains unavailable.</x:v>
       </x:c>
       <x:c r="T41" s="12" t="str">
         <x:v>Not visible in supplied photo</x:v>
@@ -3578,8 +4258,23 @@
       <x:c r="AD41" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
-    </x:row>
-    <x:row r="42" ht="90" customHeight="1">
+      <x:c r="AE41" s="12" t="str">
+        <x:v>The second volume of Shizue Sasagawa’s Aiginshū, a collection of gin’ei vocal performances. The moon-and-blossom sleeve supplies the artist and volume identification; a release date and full programme remain unverified.</x:v>
+      </x:c>
+      <x:c r="AF41" s="12" t="str">
+        <x:v>https://github.com/richardmands/record_collection/blob/main/data/reference-photos/IMG_3235.jpg</x:v>
+      </x:c>
+      <x:c r="AG41" s="12" t="str">
+        <x:v>Original sleeve (collection note)</x:v>
+      </x:c>
+      <x:c r="AH41" s="12" t="str">
+        <x:v>https://nippon.zaidan.info/seikabutsu/2005/00403/contents/0002.htm</x:v>
+      </x:c>
+      <x:c r="AI41" s="12" t="str">
+        <x:v>Nippon Foundation article</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="120" customHeight="1">
       <x:c r="A42" s="6" t="str">
         <x:v>41</x:v>
       </x:c>
@@ -3653,11 +4348,26 @@
       <x:c r="AD42" s="12" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
+      <x:c r="AE42" s="12" t="str">
+        <x:v>A nagauta performance of Shinkyoku Urashima, divided into two parts across the record’s sides. The Columbia release credits Ijūrō Yoshimura and shamisen player Eijirō Kineya.</x:v>
+      </x:c>
+      <x:c r="AF42" s="12" t="str">
+        <x:v>https://www.discogs.com/release/13923247</x:v>
+      </x:c>
+      <x:c r="AG42" s="12" t="str">
+        <x:v>Discogs release and track listing</x:v>
+      </x:c>
+      <x:c r="AH42" s="12" t="str">
+        <x:v>https://www.discogs.com/artist/2475755</x:v>
+      </x:c>
+      <x:c r="AI42" s="12" t="str">
+        <x:v>Ijūrō Yoshimura on Discogs</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R269d14054404472f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23c16bbbadd34bfe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11837,7 +12547,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0bfe17871ca4933"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8567bfd133c54917"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>